<commit_message>
Daily jobs update 2026-10-02
</commit_message>
<xml_diff>
--- a/afriworket_tracker.xlsx
+++ b/afriworket_tracker.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V201"/>
+  <dimension ref="A1:V221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17328,6 +17328,1689 @@
       <c r="V201" t="inlineStr">
         <is>
           <t>Work address: Kira</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>043d6280-bc05-4716-b609-f8b3e11b5060</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Customer service/Admission agent</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Customer Service &amp; Care</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>JUNIOR</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>1</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>Ability to Simplify Complex Ideas; Active Learning; Basic Writing; English Language; Action Oriented</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>October 6, 2026</t>
+        </is>
+      </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/043d6280-bc05-4716-b609-f8b3e11b5060</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S202" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U202" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V202" t="inlineStr">
+        <is>
+          <t>Link Education and Travel Consultant PLC
+Work address: Bisrate Gebreal</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>099ac10c-21cc-449e-bd73-19290f0babdf</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Senior Odoo ERP Finance &amp; Lead Functional Consultant</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Software Design &amp; Development</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I203" t="n">
+        <v>1</v>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>Financial And Business Management System; Financial Analysis; Financial Accounting; Training; Training Administration; Problem Solving</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>October 6, 2026</t>
+        </is>
+      </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/099ac10c-21cc-449e-bd73-19290f0babdf</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U203" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V203" t="inlineStr">
+        <is>
+          <t>360Ground
+Work address: Around 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>25252ec0-ac1d-4695-8ea4-bd62012f79f5</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Sales &amp; Promotion</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>JUNIOR</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>4</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>Customer Service</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>October 22, 2026</t>
+        </is>
+      </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/25252ec0-ac1d-4695-8ea4-bd62012f79f5</t>
+        </is>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U204" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V204" t="inlineStr">
+        <is>
+          <t>Work address: Lebu, kality, Bulbula</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>277febbe-e7c9-498f-a832-aac80d66a1ad</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales Manager</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Sales &amp; Promotion</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>EXPERT</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>2</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>Certificate</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>Strategic Selling; Customer Relationship Management; Monitor Control Command Set; Sales Performance Management; Market Access Strategy</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/277febbe-e7c9-498f-a832-aac80d66a1ad</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V205" t="inlineStr">
+        <is>
+          <t>LUCY GARMENT INDUSTRY PLC
+Work address: saris kadisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>401ee8a0-5442-4b0e-accf-4816b776d2f2</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Social Media Manager</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Multimedia Content Production</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>1</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Diploma</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Media Literacy; MediaInfo; Media Production; Media Management; Media Ethics; Media Presentations</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>October 8, 2026</t>
+        </is>
+      </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/401ee8a0-5442-4b0e-accf-4816b776d2f2</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S206" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V206" t="inlineStr">
+        <is>
+          <t>Work address: Saris</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>4122213f-6d3b-4d35-a08e-0a3b39af6359</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>sales supporter/office assistance</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Customer Service &amp; Care</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Hybrid - Full Time</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I207" t="n">
+        <v>3</v>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>Active Learning; Good Language Learner Studies; English Language; Communication</t>
+        </is>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>October 29, 2026</t>
+        </is>
+      </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/4122213f-6d3b-4d35-a08e-0a3b39af6359</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S207" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T207" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U207" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V207" t="inlineStr">
+        <is>
+          <t>Work address: goro Cambridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>56b79d30-9e63-43ac-a3f3-01a4527893a9</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Refreshed October 2, 2026</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I208" t="n">
+        <v>1</v>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>Business development; Account Management; Sales Development; Sales Management</t>
+        </is>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>October 20, 2026</t>
+        </is>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/56b79d30-9e63-43ac-a3f3-01a4527893a9</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S208" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="T208" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V208" t="inlineStr">
+        <is>
+          <t>LeuNet ICT Solutions
+Work address: Gerji/Alfoz ,</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>5d53f85f-b525-47f6-951f-759b800c4048</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Salesperson</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Sales &amp; Promotion</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>1</v>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>October 8, 2026</t>
+        </is>
+      </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/5d53f85f-b525-47f6-951f-759b800c4048</t>
+        </is>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T209" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U209" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V209" t="inlineStr">
+        <is>
+          <t>Work address: Addis Ababa . Ayat 5 Haile Gudeta building</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>63580691-5648-4d9c-8ab0-2ee6e123a9c7</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Sales person</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Sales &amp; Promotion</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I210" t="n">
+        <v>5</v>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Diploma</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>October 9, 2026</t>
+        </is>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/63580691-5648-4d9c-8ab0-2ee6e123a9c7</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T210" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U210" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V210" t="inlineStr">
+        <is>
+          <t>MERXY TRADING PLC
+Work address: Megenagna infront of israel embassy</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>6b295518-a1b3-458c-9ebc-6bc20163ecd4</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>interior and finishing Work office engineer</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Mechanical &amp; Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Hybrid - Full Time</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I211" t="n">
+        <v>4</v>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>Postgraduate Diploma</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>Safe Modes</t>
+        </is>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>October 9, 2026</t>
+        </is>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/6b295518-a1b3-458c-9ebc-6bc20163ecd4</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S211" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T211" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U211" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V211" t="inlineStr">
+        <is>
+          <t>Leo Construction
+Work address: Addisababa</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>6cf6b3b9-28f5-4488-8a00-c333f1fc13bf</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Freelance Tutor</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Tutoring, Training &amp; Mentorship</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Onsite - Freelance</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>ENTRY</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>Planning &amp; Scheduling; Mentoring Youth; Time Management; Communication; Punctuality</t>
+        </is>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>October 30, 2026</t>
+        </is>
+      </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/6cf6b3b9-28f5-4488-8a00-c333f1fc13bf</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S212" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T212" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U212" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V212" t="inlineStr">
+        <is>
+          <t>Work address: Addis Ababa</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>83e55f87-4ed2-4a94-91af-e17583ed3ece</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>outdoor sales</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Remote - Full Time</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I213" t="n">
+        <v>10</v>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>October 29, 2026</t>
+        </is>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/83e55f87-4ed2-4a94-91af-e17583ed3ece</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S213" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T213" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>8ed8871a-45d7-4d83-ac86-23f6ab16523a</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>special assistance/credit assistance</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Accounting &amp; Finance</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Hybrid - Full Time</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I214" t="n">
+        <v>1</v>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>Supportworks; Performance Management; Active Learning; Good Language Learner Studies; Action Oriented</t>
+        </is>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>October 30, 2026</t>
+        </is>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/8ed8871a-45d7-4d83-ac86-23f6ab16523a</t>
+        </is>
+      </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S214" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U214" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V214" t="inlineStr">
+        <is>
+          <t>Work address: goro Cambridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>9975f2cd-c249-4fac-a385-6a0111732c14</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Junior Stock Control Officer</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>JUNIOR</t>
+        </is>
+      </c>
+      <c r="I215" t="n">
+        <v>5</v>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>Active Learning; Patience; Action Oriented</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>October 16, 2026</t>
+        </is>
+      </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/9975f2cd-c249-4fac-a385-6a0111732c14</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S215" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T215" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U215" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V215" t="inlineStr">
+        <is>
+          <t>Minaye PLC
+Work address: Head office, torhayloch minaye building</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>b1f91dea-c864-4d00-877b-8b750eabd7eb</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Refreshed October 2, 2026</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I216" t="n">
+        <v>1</v>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>Market Research; Digital Marketing and Advertising; B2B Communication; Creative Problem-Solving; Marketing Management; Brand Management</t>
+        </is>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>October 20, 2026</t>
+        </is>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/b1f91dea-c864-4d00-877b-8b750eabd7eb</t>
+        </is>
+      </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S216" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="T216" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V216" t="inlineStr">
+        <is>
+          <t>LeuNet ICT Solutions
+Work address: Gerji/Alfoz Plaza</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>bdea7f1e-69c5-41da-872d-4ca9dc196ed4</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Safety and Quality engineer</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Security &amp; Safety</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Hybrid - Full Time</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>2</v>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Postgraduate Diploma</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>Quality Assessment</t>
+        </is>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>October 10, 2026</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/bdea7f1e-69c5-41da-872d-4ca9dc196ed4</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S217" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V217" t="inlineStr">
+        <is>
+          <t>Leo Construction
+Work address: Addisababa</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>c38afacb-cdea-4a9d-b455-09f7c511aca7</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Architecture &amp; Urban Planning</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I218" t="n">
+        <v>1</v>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>Design; Technical Drawing; 3D Graphic Design; AutoCAD; SketchUp; Problem Solving</t>
+        </is>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>October 8, 2026</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/c38afacb-cdea-4a9d-b455-09f7c511aca7</t>
+        </is>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T218" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V218" t="inlineStr">
+        <is>
+          <t>Ganador Real Estate developer
+Work address: Welo sefer , Garamulet Building 2nd Floor for more info call +2519 96759187 Note don't forget to bring your close-up photo APPLY ONLY IN PERSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>d27c73a7-372b-4541-ba4b-5030139b37cd</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Live Stream Host (Anchors)</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Multimedia Content Production</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>ENTRY</t>
+        </is>
+      </c>
+      <c r="I219" t="n">
+        <v>6</v>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>Arabic Language; English Language; Communication; Punctuality</t>
+        </is>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>October 14, 2026</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/d27c73a7-372b-4541-ba4b-5030139b37cd</t>
+        </is>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T219" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U219" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V219" t="inlineStr">
+        <is>
+          <t>Work address: Megenagna</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>d53491db-e269-430a-b93c-29f2615e188a</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Site engineer</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Construction &amp; Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Jigjiga, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I220" t="n">
+        <v>1</v>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>AutoCAD; Site Planning</t>
+        </is>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>October 8, 2026</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/d53491db-e269-430a-b93c-29f2615e188a</t>
+        </is>
+      </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T220" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U220" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V220" t="inlineStr">
+        <is>
+          <t>Work address: Gerji, Sami building</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>f7877541-54bb-473d-9f0c-d85808f3e973</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>project manager</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Construction &amp; Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Hybrid - Full Time</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>EXPERT</t>
+        </is>
+      </c>
+      <c r="I221" t="n">
+        <v>4</v>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Postgraduate Diploma</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>Civil Site Design</t>
+        </is>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>October 16, 2026</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/f7877541-54bb-473d-9f0c-d85808f3e973</t>
+        </is>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T221" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:57:30 UTC</t>
+        </is>
+      </c>
+      <c r="U221" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V221" t="inlineStr">
+        <is>
+          <t>Leo Construction
+Work address: Addisababa</t>
         </is>
       </c>
     </row>
@@ -17342,7 +19025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17391,6 +19074,25 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:58:20 UTC</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C3" t="n">
+        <v>220</v>
+      </c>
+      <c r="D3" t="n">
+        <v>40</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily jobs update 2026-10-03
</commit_message>
<xml_diff>
--- a/afriworket_tracker.xlsx
+++ b/afriworket_tracker.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V221"/>
+  <dimension ref="A1:V245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19011,6 +19011,2036 @@
         <is>
           <t>Leo Construction
 Work address: Addisababa</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>0ec79c16-257c-4ab1-b81f-3c4edb27cfbc</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Junior Accountant - ERP Trainee In Finance</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Accounting &amp; Finance</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>JUNIOR</t>
+        </is>
+      </c>
+      <c r="I222" t="n">
+        <v>1</v>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>Understanding Emotions; Ability to Simplify Complex Ideas; Ability to See Other People's Point of View; Interpersonal Communications; Communications; Training And Development</t>
+        </is>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>October 17, 2026</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/0ec79c16-257c-4ab1-b81f-3c4edb27cfbc</t>
+        </is>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T222" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U222" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V222" t="inlineStr">
+        <is>
+          <t>Tech Equations Technology
+Work address: Sarbet lidiya Bulding Office 505</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>0fcd88e2-8d98-407f-8bac-fa9f2f6fb9e6</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Senior Java Developer</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Software Design &amp; Development</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Onsite - Contractual</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I223" t="n">
+        <v>1</v>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>RabbitMQ; Kubernetes; Spring Boot; RESTful API; Java; Enterprise Application Software</t>
+        </is>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>October 9, 2026</t>
+        </is>
+      </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/0fcd88e2-8d98-407f-8bac-fa9f2f6fb9e6</t>
+        </is>
+      </c>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T223" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U223" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V223" t="inlineStr">
+        <is>
+          <t>Greenvolt Electric Vehicle Maintenance
+Work address: Addis ababa</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>1d698f82-d9cc-4027-8c9d-dd383ac9c8ab</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Senior English Language Instructor</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Teaching &amp; Education</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Onsite - Part Time</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I224" t="n">
+        <v>2</v>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>Accountability</t>
+        </is>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>October 16, 2026</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/1d698f82-d9cc-4027-8c9d-dd383ac9c8ab</t>
+        </is>
+      </c>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T224" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U224" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V224" t="inlineStr">
+        <is>
+          <t>Work address: Addis</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>25fb3df0-094f-43da-a359-1e8ce65a49c9</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Senior Computer Maintenance and Networking Expert</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Installation &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I225" t="n">
+        <v>2</v>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>Accountability</t>
+        </is>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>October 16, 2026</t>
+        </is>
+      </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/25fb3df0-094f-43da-a359-1e8ce65a49c9</t>
+        </is>
+      </c>
+      <c r="R225" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T225" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U225" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V225" t="inlineStr">
+        <is>
+          <t>Work address: Addis</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>416bd8c2-7e0b-4bc3-bb94-1a255ca0c847</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Dental Laboratory Technician</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I226" t="n">
+        <v>1</v>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Diploma</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>Teamwork; Communication</t>
+        </is>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>October 10, 2026</t>
+        </is>
+      </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/416bd8c2-7e0b-4bc3-bb94-1a255ca0c847</t>
+        </is>
+      </c>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S226" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T226" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U226" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V226" t="inlineStr">
+        <is>
+          <t>SANTE MEDICAL CENTER
+Work address: Bisrate Gebreal,Doba Building, Addis Ababa</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>4c0da52f-5604-4ce1-8116-03a359f0879a</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Food &amp; Drink Preparation / Service</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Onsite - Part Time</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I227" t="n">
+        <v>2</v>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>October 7, 2026</t>
+        </is>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/4c0da52f-5604-4ce1-8116-03a359f0879a</t>
+        </is>
+      </c>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T227" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U227" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V227" t="inlineStr">
+        <is>
+          <t>Work address: Bole around moenco</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>558cc55e-42f2-4c36-b831-02aaf5e24376</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Architect- Furniture &amp; Interior Design</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Architecture &amp; Urban Planning</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Onsite - Contractual</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I228" t="n">
+        <v>1</v>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>Detail Oriented; Furniture Design; Interior Design; Ability To Meet Deadlines; Creativity; Communication</t>
+        </is>
+      </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>October 27, 2026</t>
+        </is>
+      </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/558cc55e-42f2-4c36-b831-02aaf5e24376</t>
+        </is>
+      </c>
+      <c r="R228" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S228" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T228" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U228" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V228" t="inlineStr">
+        <is>
+          <t>Work address: Ahemed Business Center, Ledeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>6447c76b-84d7-447c-b036-7acfa861ecc5</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Senior Graphic Design and Video Editing Instructor</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Creative Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Onsite - Part Time</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I229" t="n">
+        <v>3</v>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>Accountability</t>
+        </is>
+      </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>October 16, 2026</t>
+        </is>
+      </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/6447c76b-84d7-447c-b036-7acfa861ecc5</t>
+        </is>
+      </c>
+      <c r="R229" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S229" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T229" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U229" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V229" t="inlineStr">
+        <is>
+          <t>Work address: Addis</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>7059e467-b091-4379-8e2b-7125d48348fe</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Outdoor salesperson</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Sales &amp; Promotion</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Hybrid - Part Time</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I230" t="n">
+        <v>20</v>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>High School</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>Marketing Intelligence; Marketing Communication; Sales Intelligence</t>
+        </is>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>October 31, 2026</t>
+        </is>
+      </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/7059e467-b091-4379-8e2b-7125d48348fe</t>
+        </is>
+      </c>
+      <c r="R230" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S230" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T230" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U230" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V230" t="inlineStr">
+        <is>
+          <t>INFINITY BUSINESS GROUP PLC
+Work address: Bole Medhanialem Mall 10th floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>71801947-43f2-4fac-8c57-d62293cd868f</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Reception and Sales</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Sales &amp; Promotion</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I231" t="n">
+        <v>4</v>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>Accountability</t>
+        </is>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>October 16, 2026</t>
+        </is>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/71801947-43f2-4fac-8c57-d62293cd868f</t>
+        </is>
+      </c>
+      <c r="R231" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T231" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U231" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V231" t="inlineStr">
+        <is>
+          <t>Work address: Addis</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>74459e37-6f58-4abb-8b54-077c237d42a2</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>General foreman</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Construction &amp; Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Jimma, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Onsite - Contractual</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I232" t="n">
+        <v>1</v>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Diploma</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>Leadership</t>
+        </is>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>October 6, 2026</t>
+        </is>
+      </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/74459e37-6f58-4abb-8b54-077c237d42a2</t>
+        </is>
+      </c>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T232" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U232" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V232" t="inlineStr">
+        <is>
+          <t>Work address: Jimma city</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>7def9265-e1e2-4f11-b296-313f00a2b834</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Refreshed October 3, 2026</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Customer Service &amp; Care</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>JUNIOR</t>
+        </is>
+      </c>
+      <c r="I233" t="n">
+        <v>1</v>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>October 25, 2026</t>
+        </is>
+      </c>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/7def9265-e1e2-4f11-b296-313f00a2b834</t>
+        </is>
+      </c>
+      <c r="R233" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S233" t="inlineStr">
+        <is>
+          <t>September 27, 2026</t>
+        </is>
+      </c>
+      <c r="T233" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U233" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V233" t="inlineStr">
+        <is>
+          <t>Work address: Gerji mebrat hail</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>85fa9f56-fbb1-416a-b71e-646e6cffeca2</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Graphics designer and secretery</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Multimedia Content Production</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I234" t="n">
+        <v>2</v>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>Not Required</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>Adaptability &amp; Resilience</t>
+        </is>
+      </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/85fa9f56-fbb1-416a-b71e-646e6cffeca2</t>
+        </is>
+      </c>
+      <c r="R234" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T234" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U234" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V234" t="inlineStr">
+        <is>
+          <t>Wibet Print Press and Branding
+Work address: Kera(ቄራ) downtown and Ayertena (አየርጤና)</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>887f7490-4993-4c9e-a25d-d3a6bcea2591</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Nanny</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Onsite - Part Time</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>Certificate</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>October 17, 2026</t>
+        </is>
+      </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/887f7490-4993-4c9e-a25d-d3a6bcea2591</t>
+        </is>
+      </c>
+      <c r="R235" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S235" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T235" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U235" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V235" t="inlineStr">
+        <is>
+          <t>Keyborn studio
+Work address: Bole , adisu stadium, Behind Ag grace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>8a7c5b44-231d-495b-ac11-652b3c8b554a</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>የአቤቱታ ክትትል እና ቅሬታ ሰሚ ባለሞያ</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Customer Service &amp; Care</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I236" t="n">
+        <v>1</v>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>Legal Knowledge</t>
+        </is>
+      </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>October 16, 2026</t>
+        </is>
+      </c>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/8a7c5b44-231d-495b-ac11-652b3c8b554a</t>
+        </is>
+      </c>
+      <c r="R236" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S236" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T236" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U236" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V236" t="inlineStr">
+        <is>
+          <t>Work address: Oraeale</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>a9b3f39b-b521-41c6-9d88-4ed3ecdd66e9</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Female Special Needs Education (SNE) Teacher</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Teaching &amp; Education</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>JUNIOR</t>
+        </is>
+      </c>
+      <c r="I237" t="n">
+        <v>2</v>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>Human Health Risk Assessment; Psychological Counseling; Creative Problem-Solving; Adaptability &amp; Resilience</t>
+        </is>
+      </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>October 10, 2026</t>
+        </is>
+      </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/a9b3f39b-b521-41c6-9d88-4ed3ecdd66e9</t>
+        </is>
+      </c>
+      <c r="R237" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S237" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T237" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U237" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V237" t="inlineStr">
+        <is>
+          <t>Zoma museum plc
+Work address: Zoma Museum Head Office &amp; Moving to locations</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>aef04e21-7d9a-4a24-bd1f-d70fa44f9aa0</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Software Developer</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Software Design &amp; Development</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I238" t="n">
+        <v>3</v>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>Spring Boot; Java; C#</t>
+        </is>
+      </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>October 7, 2026</t>
+        </is>
+      </c>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/aef04e21-7d9a-4a24-bd1f-d70fa44f9aa0</t>
+        </is>
+      </c>
+      <c r="R238" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T238" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U238" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V238" t="inlineStr">
+        <is>
+          <t>Work address: Addis Abeba Mexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>b0164b21-e528-4581-bb70-4b517befc8e0</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Senior HR Admin and Manager</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Human Resource &amp; Talent Management</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>SENIOR</t>
+        </is>
+      </c>
+      <c r="I239" t="n">
+        <v>1</v>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>Management Control Systems</t>
+        </is>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>October 22, 2026</t>
+        </is>
+      </c>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/b0164b21-e528-4581-bb70-4b517befc8e0</t>
+        </is>
+      </c>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T239" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U239" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V239" t="inlineStr">
+        <is>
+          <t>Barkonal Travel Agent
+Work address: 22 AREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>ba907cce-eb2e-418c-8918-acd076a99a60</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Dental clinic Reception</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Customer Service &amp; Care</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>JUNIOR</t>
+        </is>
+      </c>
+      <c r="I240" t="n">
+        <v>1</v>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>Computer Keyboards</t>
+        </is>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>October 22, 2026</t>
+        </is>
+      </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/ba907cce-eb2e-418c-8918-acd076a99a60</t>
+        </is>
+      </c>
+      <c r="R240" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S240" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T240" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U240" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V240" t="inlineStr">
+        <is>
+          <t>Work address: Hayahulet</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>d66a95bd-3064-4e85-ad6f-a46f9d901db3</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Customer Service Representative- Seasonal</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Customer Service &amp; Care</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Remote - Full Time</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I241" t="n">
+        <v>2</v>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>October 15, 2026</t>
+        </is>
+      </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/d66a95bd-3064-4e85-ad6f-a46f9d901db3</t>
+        </is>
+      </c>
+      <c r="R241" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S241" t="inlineStr">
+        <is>
+          <t>October 2, 2026</t>
+        </is>
+      </c>
+      <c r="T241" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U241" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>e1b989af-0f2b-4de5-80d5-e73a40488b45</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Real estate sales consultant</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Sales &amp; Promotion</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>JUNIOR</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>Creative Thinking; Creativity; Communication</t>
+        </is>
+      </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>October 4, 2026</t>
+        </is>
+      </c>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/e1b989af-0f2b-4de5-80d5-e73a40488b45</t>
+        </is>
+      </c>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S242" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T242" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U242" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V242" t="inlineStr">
+        <is>
+          <t>Reliable Homes Business and Marketing
+Work address: Summit</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>e9fd456f-5cdd-415d-9ad8-8f4ed4e3ddf9</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Sales and Customer Relations</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Advisory &amp; Consultancy</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Hybrid - Full Time</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I243" t="n">
+        <v>5</v>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>Presentation Skills; Digital Media Production; Communication; Online Marketing</t>
+        </is>
+      </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>October 10, 2026</t>
+        </is>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/e9fd456f-5cdd-415d-9ad8-8f4ed4e3ddf9</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S243" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T243" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U243" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V243" t="inlineStr">
+        <is>
+          <t>HMR Business Solutions PLC
+Work address: Addis Ababa</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>f8e86424-9732-46ec-82cd-dfb07a4eb8b2</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Secretary &amp; Accountant</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Private Client</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Accounting &amp; Finance</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>JUNIOR</t>
+        </is>
+      </c>
+      <c r="I244" t="n">
+        <v>2</v>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>Microsoft 365; Integrity Management; Organisational Policies; Finance; Confident Communicator; Communication</t>
+        </is>
+      </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>October 23, 2026</t>
+        </is>
+      </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/f8e86424-9732-46ec-82cd-dfb07a4eb8b2</t>
+        </is>
+      </c>
+      <c r="R244" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S244" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T244" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U244" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V244" t="inlineStr">
+        <is>
+          <t>Work address: Dembel</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>fe3bc38f-0554-4968-a77e-81e2127b7bf8</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Office Engineer(Tender)</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Construction &amp; Civil Engineering</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Addis Ababa, Ethiopia</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Onsite - Full Time</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>INTERMEDIATE</t>
+        </is>
+      </c>
+      <c r="I245" t="n">
+        <v>2</v>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Bachelor’s Degree</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>Computer Assisted Audit Tools And Techniques; Scheduling; Qualification Protocols IQ/OQ/PQ; Organization</t>
+        </is>
+      </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>October 9, 2026</t>
+        </is>
+      </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>https://afriworket.com/jobs/fe3bc38f-0554-4968-a77e-81e2127b7bf8</t>
+        </is>
+      </c>
+      <c r="R245" t="inlineStr">
+        <is>
+          <t>Afriworket</t>
+        </is>
+      </c>
+      <c r="S245" t="inlineStr">
+        <is>
+          <t>October 3, 2026</t>
+        </is>
+      </c>
+      <c r="T245" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:22 UTC</t>
+        </is>
+      </c>
+      <c r="U245" t="inlineStr">
+        <is>
+          <t>detail_page</t>
+        </is>
+      </c>
+      <c r="V245" t="inlineStr">
+        <is>
+          <t>Zota Engineering PLC
+Work address: CMC(figa)</t>
         </is>
       </c>
     </row>
@@ -19025,7 +21055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19093,6 +21123,25 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-03 10:53:54 UTC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>24</v>
+      </c>
+      <c r="C4" t="n">
+        <v>244</v>
+      </c>
+      <c r="D4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>